<commit_message>
Daily check: sleeve badge option vs team/league on all sites
parse_badges reads each badge option with its pictures (PPOM data-label
on CFS, Extra Product Options label + picture alt/filename on KFK, RFS,
RFK; regex only, matching BeautifulSoup on 128 sample pages).
sleeve_badge.py is the copy of football-qa-tools CFS/sleeve_badge.py.
Wrong team/league = CAO, option/picture/description wording = Trung
binh, reviews needing a person = Thap.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0149ELLgZdjaY7wRsdGLp26m
</commit_message>
<xml_diff>
--- a/listing-monitor/reports/2026-10-28/qa_2026-10-28.xlsx
+++ b/listing-monitor/reports/2026-10-28/qa_2026-10-28.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="KFK" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="RFS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="RFK" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CFS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cần xác nhận" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KFK" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFK" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cần xác nhận" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KFK'!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'KFK'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RFS'!$A$1:$N$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RFK'!$A$1:$N$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CFS'!$A$1:$N$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CFS'!$A$1:$N$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -65,17 +65,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2E3E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
   </fills>
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tạo lúc 2026-10-28 23:37. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
+          <t>Tạo lúc 2026-10-29 08:24. Mức độ: Cao = sai thông tin / gây confuse khách và Google; Trung bình = cần sửa; Thấp = nên sửa.</t>
         </is>
       </c>
     </row>
@@ -544,16 +544,16 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -616,19 +616,19 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -674,14 +674,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Christmas campaign</t>
+          <t>Sai Home/Away/Third</t>
         </is>
       </c>
       <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
         <v>2</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -696,14 +696,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sai Home/Away/Third</t>
+          <t>Sai tất (socks)</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>0</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>0</v>
@@ -712,17 +712,17 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sai tất (socks)</t>
+          <t>SEO tên cầu thủ</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -731,7 +731,7 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>2</v>
@@ -740,14 +740,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SEO tên cầu thủ</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
@@ -756,20 +756,20 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Sai loại Shirt/Kit</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -778,17 +778,17 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sai loại Shirt/Kit</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
@@ -797,10 +797,10 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -828,14 +828,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Club bị report (KFK)</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
@@ -844,20 +844,20 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Club bị report (KFK)</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
@@ -866,17 +866,17 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
         <v>2</v>
@@ -888,7 +888,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -902,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -996,7 +996,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -1015,22 +1015,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Christmas campaign</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Listing đăng trong đợt Christmas nhưng chưa có ảnh AI Christmas (không có ảnh nào tên/alt chứa Xmas/Christmas)</t>
+          <t>'Badge' (...nd number 17 already applied. Badge options: La Liga Champions sl...)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh AI Christmas (đặt tên file/alt có chữ Xmas)</t>
+          <t>Badge -&gt; chest detail</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -1050,47 +1050,47 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
-        <v>265479</v>
+        <v>265465</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KFK_BA_HO_KD_GORDON 17_26/27</t>
+          <t>KFK_BA_AW_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Barcelona Home Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
+          <t>Barcelona Away Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Christmas campaign</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Listing đăng trong đợt Christmas nhưng chưa có ảnh AI Christmas (không có ảnh nào tên/alt chứa Xmas/Christmas)</t>
+          <t>1/6 ảnh không có alt text</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Thêm ảnh AI Christmas (đặt tên file/alt có chữ Xmas)</t>
+          <t>Thêm alt text riêng cho từng ảnh</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/barcelona-home-kids-football-kit-2026-27-gordon-17/</t>
+          <t>https://kidsfootballkit.co.uk/product/barcelona-away-kids-football-kit-2026-27-gordon-17/</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -1102,7 +1102,7 @@
       <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
@@ -1123,22 +1123,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>SEO tên cầu thủ</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Tên sản phẩm</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>'Badge' (...nd number 17 already applied. Badge options: La Liga Champions sl...)</t>
+          <t>Tên cầu thủ đang ở cuối tên ('GORDON 17'): các URL cùng mẫu áo trùng phần đầu</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Badge -&gt; chest detail</t>
+          <t>Đổi theo format: [Club] [PLAYER] [Số] [Home/Away] [Men/Kids] ... (giữ nguyên slug)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -1156,49 +1156,49 @@
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>265465</v>
+        <v>265479</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KFK_BA_AW_KD_GORDON 17_26/27</t>
+          <t>KFK_BA_HO_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Barcelona Away Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
+          <t>Barcelona Home Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SEO tên cầu thủ</t>
+          <t>Words to Avoid</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tên sản phẩm</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Tên cầu thủ đang ở cuối tên ('GORDON 17'): các URL cùng mẫu áo trùng phần đầu</t>
+          <t>'Badge' (...umber 17 applied to the back. Badge options: La Liga Champions sl...)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Đổi theo format: [Club] [PLAYER] [Số] [Home/Away] [Men/Kids] ... (giữ nguyên slug)</t>
+          <t>Badge -&gt; chest detail</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/barcelona-away-kids-football-kit-2026-27-gordon-17/</t>
+          <t>https://kidsfootballkit.co.uk/product/barcelona-home-kids-football-kit-2026-27-gordon-17/</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -1210,7 +1210,7 @@
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
@@ -1231,22 +1231,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Words to Avoid</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Alt text</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>'Badge' (...umber 17 applied to the back. Badge options: La Liga Champions sl...)</t>
+          <t>1/6 ảnh không có alt text</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Badge -&gt; chest detail</t>
+          <t>Thêm alt text riêng cho từng ảnh</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -1264,7 +1264,7 @@
       <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
@@ -1318,7 +1318,7 @@
       <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
@@ -1372,7 +1372,7 @@
       <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -1426,7 +1426,7 @@
       <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -1480,7 +1480,7 @@
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -1534,49 +1534,49 @@
       <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>265479</v>
+        <v>265465</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KFK_BA_HO_KD_GORDON 17_26/27</t>
+          <t>KFK_BA_AW_KD_GORDON 17_26/27</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Barcelona Home Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
+          <t>Barcelona Away Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SEO</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SEO title</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Rút gọn</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>https://kidsfootballkit.co.uk/product/barcelona-home-kids-football-kit-2026-27-gordon-17/</t>
+          <t>https://kidsfootballkit.co.uk/product/barcelona-away-kids-football-kit-2026-27-gordon-17/</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1588,7 +1588,7 @@
       <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -1609,22 +1609,22 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Club bị report (KFK)</t>
+          <t>SEO</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ảnh</t>
+          <t>SEO title</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Barcelona: 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
+          <t>SEO title dài 66 ký tự (nên &lt;= 60)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Check blur logo</t>
+          <t>Rút gọn</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1642,7 +1642,7 @@
       <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -1663,22 +1663,22 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Club bị report (KFK)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>SKU (Google)</t>
+          <t>Ảnh</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>SKU 'KFK_BA_HO_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+          <t>Barcelona: 'Published (blurred logo)', nhớ kiểm tra logo đã blur trên ảnh</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+          <t>Check blur logo</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1695,8 +1695,116 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="n">
+        <v>265479</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KFK_BA_HO_KD_GORDON 17_26/27</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Barcelona Home Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>SKU (Google)</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>SKU 'KFK_BA_HO_KD_GORDON 17_26/27' có dấu cách hoặc ký tự đặc biệt: Google Merchant không nhận</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Dùng chữ không dấu, số, - hoặc _ (vd FERRAN-9)</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://kidsfootballkit.co.uk/product/barcelona-home-kids-football-kit-2026-27-gordon-17/</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>265479</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>KFK_BA_HO_KD_GORDON 17_26/27</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Barcelona Home Kids Football Kit 2026/27 – GORDON 17 (With socks)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Sleeve badge</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Option badge</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Cần người check</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://kidsfootballkit.co.uk/product/barcelona-home-kids-football-kit-2026-27-gordon-17/</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N14"/>
+  <autoFilter ref="A1:N16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -1724,6 +1832,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1827,7 +1939,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Cao</t>
         </is>
@@ -1881,7 +1993,7 @@
       <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Cao</t>
         </is>
@@ -1935,7 +2047,7 @@
       <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
@@ -1989,7 +2101,7 @@
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
@@ -2043,7 +2155,7 @@
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Trung bình</t>
         </is>
@@ -2097,7 +2209,7 @@
       <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -2151,7 +2263,7 @@
       <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -2205,7 +2317,7 @@
       <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -2259,7 +2371,7 @@
       <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -2313,7 +2425,7 @@
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -2367,7 +2479,7 @@
       <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
@@ -2559,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2651,7 +2763,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Cao</t>
         </is>
@@ -2707,7 +2819,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -2726,22 +2838,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sai Home/Away/Third</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Tên là third nhưng đầu description ghi away: For Inter Milan’s 2026/27 season, this away football kit comes in white. Kit Facts Team: Inter Milan Se...</t>
+          <t>Description ghi sleeve badge "Serie A can be added" nhưng option là Serie A (champion) (lệch chữ Champions) → sửa cho khớp.</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Sửa description (có thể copy từ listing khác)</t>
+          <t>Thống nhất có/không chữ Champions giữa option và description</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -2759,49 +2871,49 @@
       <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Cao</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>84891</v>
+        <v>84836</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CFS_ITM_TH_KD_No_26/27</t>
+          <t>CFS_BAR_AWLV_KD_No_26/27</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Inter Milan Third Kids Cheap Football Kit 2026/27</t>
+          <t>Barcelona Away Kids Cheap Football Kit 2026/27 Long Sleeve</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sai Home/Away/Third</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Description ghi Kit: Away, nhưng tên là third</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Sửa ô Kit trong description</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-milan-third-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-away-kids-cheap-football-kit-2026-27-long-sleeve/</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -2813,49 +2925,49 @@
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Cao</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="n">
-        <v>84891</v>
+        <v>84847</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CFS_ITM_TH_KD_No_26/27</t>
+          <t>CFS_BAR_HOLV_KD_No_26/27</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Inter Milan Third Kids Cheap Football Kit 2026/27</t>
+          <t>Barcelona Home Kids Cheap Football Kit 2026/27 Long Sleeve</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Sai Home/Away/Third</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Trang sản phẩm (option / tab / description)</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Tên là third nhưng trang ghi: "For Inter Milan’s 2026/27 season, this away football kit comes in white."</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Sửa mọi chỗ ghi sai loại áo (option personalisation, tên biến thể, description, tab)</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-milan-third-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-home-kids-cheap-football-kit-2026-27-long-sleeve/</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -2867,49 +2979,49 @@
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Cao</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>84891</v>
+        <v>84858</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CFS_ITM_TH_KD_No_26/27</t>
+          <t>CFS_BAR_OrangeGK_KD_No_26/27</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Inter Milan Third Kids Cheap Football Kit 2026/27</t>
+          <t>Barcelona Orange Goalkeeper Kids Cheap Football Kit 2026/27</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sai tất (socks)</t>
+          <t>Sleeve badge</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Trang sản phẩm (option / tab / description)</t>
+          <t>Option badge</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Listing No Socks nhưng trang ghi: "1 shirt, matching shorts and socks."</t>
+          <t>Chưa có dữ liệu vô địch La Liga 2025/26 → cần người check badge champion của Barcelona.</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Sửa cho khớp có/không có tất</t>
+          <t>Cần người check</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>https://cheapfootballshirts.com/product/inter-milan-third-kids-cheap-football-kit-2026-27/</t>
+          <t>https://cheapfootballshirts.com/product/barcelona-orange-goalkeeper-kids-cheap-football-kit-2026-27/</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -2920,8 +3032,62 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="n">
+        <v>84891</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CFS_ITM_TH_KD_No_26/27</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Inter Milan Third Kids Cheap Football Kit 2026/27</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Sleeve badge</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Option badge</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Chưa có dữ liệu vô địch Serie A 2025/26 → cần người check badge champion của Inter Milan.</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Cần người check</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://cheapfootballshirts.com/product/inter-milan-third-kids-cheap-football-kit-2026-27/</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Mở</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:N7"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId2"/>
@@ -2933,6 +3099,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>